<commit_message>
Add sales performance dashboard Excel file
</commit_message>
<xml_diff>
--- a/Sales_Performance_Dashboard.xlsx
+++ b/Sales_Performance_Dashboard.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F8813A-6ED6-4FF5-B038-4B4992D10ABF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBB4CB8-7A01-4EC1-95DA-A394381F0292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="8" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="8" r:id="rId1"/>
     <sheet name="Row data" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
@@ -750,9 +750,6 @@
     <t xml:space="preserve">          Monthly Sales Trend</t>
   </si>
   <si>
-    <t>Target Achievement %  by Salesperson</t>
-  </si>
-  <si>
     <t xml:space="preserve">Regional Sales Performance </t>
   </si>
   <si>
@@ -760,6 +757,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Target Achievement  by Salesperson</t>
   </si>
 </sst>
 </file>
@@ -1371,6 +1371,29 @@
       <c:pivotFmt>
         <c:idx val="8"/>
         <c:spPr>
+          <a:gradFill rotWithShape="1">
+            <a:gsLst>
+              <a:gs pos="0">
+                <a:schemeClr val="accent1">
+                  <a:shade val="51000"/>
+                  <a:satMod val="130000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="80000">
+                <a:schemeClr val="accent1">
+                  <a:shade val="93000"/>
+                  <a:satMod val="130000"/>
+                </a:schemeClr>
+              </a:gs>
+              <a:gs pos="100000">
+                <a:schemeClr val="accent1">
+                  <a:shade val="94000"/>
+                  <a:satMod val="135000"/>
+                </a:schemeClr>
+              </a:gs>
+            </a:gsLst>
+            <a:lin ang="16200000" scaled="0"/>
+          </a:gradFill>
           <a:ln w="34925" cap="rnd">
             <a:solidFill>
               <a:schemeClr val="accent1"/>
@@ -1384,6 +1407,17 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </c:spPr>
         <c:marker>
           <c:symbol val="circle"/>
@@ -8825,8 +8859,8 @@
       <xdr:row>36</xdr:row>
       <xdr:rowOff>5907</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="33" name="City 7">
@@ -8849,7 +8883,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -12356,7 +12390,7 @@
       <c r="AI1" s="6"/>
       <c r="AJ1" s="6"/>
       <c r="AK1" s="14" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="AL1" s="5"/>
       <c r="AM1" s="5"/>
@@ -13373,7 +13407,7 @@
       <c r="M25" s="10"/>
       <c r="N25" s="10"/>
       <c r="O25" s="11" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="P25" s="10"/>
       <c r="Q25" s="10"/>
@@ -13926,7 +13960,7 @@
       <c r="C38" s="10"/>
       <c r="D38" s="10"/>
       <c r="E38" s="11" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F38" s="10"/>
       <c r="G38" s="10"/>
@@ -13941,7 +13975,7 @@
       <c r="P38" s="10"/>
       <c r="Q38" s="10"/>
       <c r="R38" s="11" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="S38" s="10"/>
       <c r="T38" s="10"/>

</xml_diff>